<commit_message>
Fix fruit/ingredient parsing, salmon limit, soup names
</commit_message>
<xml_diff>
--- a/Ingredient.xlsx
+++ b/Ingredient.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cheong Hengq\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cheong Hengq\Desktop\Cheong Hengq\Learnings\Python\Meal2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{046CB88F-3783-4759-A3CC-BD075752D176}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF315159-AF93-4AE4-AC02-CBE0A5881ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{1B3A883A-8798-493A-91E7-EDD802F8FD64}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="94">
   <si>
     <t>Meat / Protein</t>
   </si>
@@ -228,9 +228,6 @@
     <t>Herbal Chicken</t>
   </si>
   <si>
-    <t>Tofu Minced Pork</t>
-  </si>
-  <si>
     <t>Tofu egg</t>
   </si>
   <si>
@@ -246,21 +243,6 @@
     <t>Vegetable</t>
   </si>
   <si>
-    <t>Winter Melon</t>
-  </si>
-  <si>
-    <t>ABC</t>
-  </si>
-  <si>
-    <t>Si Shen</t>
-  </si>
-  <si>
-    <t>Liu Wei</t>
-  </si>
-  <si>
-    <t>Dun Ji Tang</t>
-  </si>
-  <si>
     <t>Ingredient 1</t>
   </si>
   <si>
@@ -270,10 +252,70 @@
     <t>Ingredient 3</t>
   </si>
   <si>
-    <t>Ingredient 4</t>
-  </si>
-  <si>
     <t>Ingredients</t>
+  </si>
+  <si>
+    <t>Raspberry</t>
+  </si>
+  <si>
+    <t>Blackberries</t>
+  </si>
+  <si>
+    <t>Chicken Tofu</t>
+  </si>
+  <si>
+    <t>Chicken breast</t>
+  </si>
+  <si>
+    <t>Sardine Tofu</t>
+  </si>
+  <si>
+    <t>Prawn</t>
+  </si>
+  <si>
+    <t>Prawn Pasta</t>
+  </si>
+  <si>
+    <t>Strawberry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avocado </t>
+  </si>
+  <si>
+    <t>Avocado Banana</t>
+  </si>
+  <si>
+    <t>Avocado</t>
+  </si>
+  <si>
+    <t>Milk</t>
+  </si>
+  <si>
+    <t>Black bean Soup</t>
+  </si>
+  <si>
+    <t>Winter Melon Soup</t>
+  </si>
+  <si>
+    <t>ABC Soup</t>
+  </si>
+  <si>
+    <t>Si Shen Soup</t>
+  </si>
+  <si>
+    <t>Liu Wei Soup</t>
+  </si>
+  <si>
+    <t>Old cucumber Soup</t>
+  </si>
+  <si>
+    <t>Dun Ji Tang Soup</t>
+  </si>
+  <si>
+    <t>Chicken bone Soup</t>
+  </si>
+  <si>
+    <t>Fish bone Soup</t>
   </si>
 </sst>
 </file>
@@ -640,22 +682,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{598DA40B-AA60-4861-8BE5-2B96676537CD}">
-  <dimension ref="B3:H51"/>
+  <dimension ref="B3:H55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.85546875" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.42578125" customWidth="1"/>
     <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.28515625" customWidth="1"/>
-    <col min="6" max="6" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13" customWidth="1"/>
     <col min="7" max="7" width="13.140625" customWidth="1"/>
     <col min="8" max="8" width="16.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
@@ -809,6 +851,9 @@
       <c r="E11" t="s">
         <v>35</v>
       </c>
+      <c r="F11" t="s">
+        <v>73</v>
+      </c>
       <c r="H11" t="s">
         <v>55</v>
       </c>
@@ -823,6 +868,9 @@
       <c r="D12" t="s">
         <v>26</v>
       </c>
+      <c r="F12" t="s">
+        <v>74</v>
+      </c>
       <c r="H12" t="s">
         <v>56</v>
       </c>
@@ -837,6 +885,9 @@
       <c r="D13" t="s">
         <v>27</v>
       </c>
+      <c r="F13" t="s">
+        <v>80</v>
+      </c>
       <c r="H13" t="s">
         <v>57</v>
       </c>
@@ -848,6 +899,9 @@
       <c r="D14" t="s">
         <v>28</v>
       </c>
+      <c r="F14" t="s">
+        <v>81</v>
+      </c>
       <c r="H14" t="s">
         <v>58</v>
       </c>
@@ -863,22 +917,25 @@
         <v>59</v>
       </c>
     </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>78</v>
+      </c>
+    </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
         <v>60</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>78</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="F19" s="1"/>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
@@ -887,15 +944,18 @@
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="C21" t="s">
-        <v>3</v>
+        <v>76</v>
+      </c>
+      <c r="D21" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C22" t="s">
         <v>3</v>
@@ -903,18 +963,15 @@
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C23" t="s">
-        <v>1</v>
-      </c>
-      <c r="D23" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C24" t="s">
         <v>8</v>
@@ -925,7 +982,7 @@
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C25" t="s">
         <v>4</v>
@@ -936,7 +993,7 @@
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C26" t="s">
         <v>5</v>
@@ -958,83 +1015,63 @@
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="C28" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
+        <v>67</v>
+      </c>
+      <c r="C29" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>69</v>
+        <v>79</v>
+      </c>
+      <c r="C30" t="s">
+        <v>78</v>
+      </c>
+      <c r="D30" t="s">
+        <v>46</v>
+      </c>
+      <c r="E30" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B31" t="str">
-        <f>C31</f>
+      <c r="B31" t="s">
+        <v>82</v>
+      </c>
+      <c r="C31" t="s">
+        <v>83</v>
+      </c>
+      <c r="D31" t="s">
+        <v>38</v>
+      </c>
+      <c r="E31" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B35" t="str">
+        <f>C35</f>
         <v>Spinach</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C35" t="s">
         <v>15</v>
-      </c>
-      <c r="D31" t="s">
-        <v>23</v>
-      </c>
-      <c r="E31" t="s">
-        <v>21</v>
-      </c>
-      <c r="F31" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B32" t="s">
-        <v>19</v>
-      </c>
-      <c r="C32" t="s">
-        <v>19</v>
-      </c>
-      <c r="D32" t="s">
-        <v>27</v>
-      </c>
-      <c r="E32" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B33" t="s">
-        <v>12</v>
-      </c>
-      <c r="C33" t="s">
-        <v>12</v>
-      </c>
-      <c r="D33" t="s">
-        <v>23</v>
-      </c>
-      <c r="E33" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B34" t="s">
-        <v>13</v>
-      </c>
-      <c r="C34" t="s">
-        <v>13</v>
-      </c>
-      <c r="D34" t="s">
-        <v>23</v>
-      </c>
-      <c r="E34" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B35" t="s">
-        <v>14</v>
-      </c>
-      <c r="C35" t="s">
-        <v>14</v>
       </c>
       <c r="D35" t="s">
         <v>23</v>
@@ -1043,26 +1080,26 @@
         <v>21</v>
       </c>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C36" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D36" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E36" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="37" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C37" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D37" t="s">
         <v>23</v>
@@ -1071,12 +1108,12 @@
         <v>21</v>
       </c>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C38" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D38" t="s">
         <v>23</v>
@@ -1085,12 +1122,12 @@
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C39" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D39" t="s">
         <v>23</v>
@@ -1099,138 +1136,194 @@
         <v>21</v>
       </c>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>15</v>
+      </c>
+      <c r="C40" t="s">
+        <v>15</v>
+      </c>
+      <c r="D40" t="s">
+        <v>23</v>
+      </c>
+      <c r="E40" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="41" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B41" t="s">
+        <v>16</v>
+      </c>
+      <c r="C41" t="s">
+        <v>16</v>
+      </c>
+      <c r="D41" t="s">
+        <v>23</v>
+      </c>
+      <c r="E41" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
+        <v>17</v>
+      </c>
+      <c r="C42" t="s">
+        <v>17</v>
+      </c>
+      <c r="D42" t="s">
+        <v>23</v>
+      </c>
+      <c r="E42" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="43" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B43" t="s">
+        <v>18</v>
+      </c>
+      <c r="C43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D43" t="s">
+        <v>23</v>
+      </c>
+      <c r="E43" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B46" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B43" t="s">
-        <v>53</v>
-      </c>
-      <c r="C43" t="s">
-        <v>50</v>
-      </c>
-      <c r="D43" t="s">
-        <v>53</v>
-      </c>
-      <c r="E43" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B44" t="s">
-        <v>70</v>
-      </c>
-      <c r="C44" t="s">
-        <v>50</v>
-      </c>
-      <c r="D44" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B45" t="s">
-        <v>71</v>
-      </c>
-      <c r="C45" t="s">
-        <v>50</v>
-      </c>
-      <c r="D45" t="s">
-        <v>23</v>
-      </c>
-      <c r="E45" t="s">
-        <v>43</v>
-      </c>
-      <c r="F45" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B46" t="s">
-        <v>72</v>
-      </c>
-      <c r="C46" t="s">
-        <v>50</v>
-      </c>
-      <c r="D46" t="s">
-        <v>23</v>
-      </c>
-      <c r="E46" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="C47" t="s">
         <v>50</v>
       </c>
       <c r="D47" t="s">
-        <v>23</v>
+        <v>53</v>
       </c>
       <c r="E47" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="48" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
-        <v>56</v>
+        <v>86</v>
       </c>
       <c r="C48" t="s">
         <v>50</v>
       </c>
       <c r="D48" t="s">
-        <v>23</v>
-      </c>
-      <c r="E48" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="49" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B49" t="s">
+        <v>87</v>
+      </c>
+      <c r="C49" t="s">
+        <v>50</v>
+      </c>
+      <c r="D49" t="s">
+        <v>23</v>
+      </c>
+      <c r="E49" t="s">
+        <v>43</v>
+      </c>
+      <c r="F49" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="50" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B50" t="s">
+        <v>88</v>
+      </c>
+      <c r="C50" t="s">
+        <v>50</v>
+      </c>
+      <c r="D50" t="s">
+        <v>23</v>
+      </c>
+      <c r="E50" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="51" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B51" t="s">
+        <v>89</v>
+      </c>
+      <c r="C51" t="s">
+        <v>50</v>
+      </c>
+      <c r="D51" t="s">
+        <v>23</v>
+      </c>
+      <c r="E51" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="52" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B52" t="s">
+        <v>90</v>
+      </c>
+      <c r="C52" t="s">
+        <v>50</v>
+      </c>
+      <c r="D52" t="s">
+        <v>23</v>
+      </c>
+      <c r="E52" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="49" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B49" t="s">
-        <v>74</v>
-      </c>
-      <c r="C49" t="s">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B53" t="s">
+        <v>91</v>
+      </c>
+      <c r="C53" t="s">
         <v>10</v>
       </c>
-      <c r="D49" t="s">
-        <v>23</v>
-      </c>
-      <c r="E49" t="s">
+      <c r="D53" t="s">
+        <v>23</v>
+      </c>
+      <c r="E53" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="50" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B50" t="s">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B54" t="s">
+        <v>92</v>
+      </c>
+      <c r="C54" t="s">
         <v>51</v>
       </c>
-      <c r="C50" t="s">
-        <v>51</v>
-      </c>
-      <c r="D50" t="s">
+      <c r="D54" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="51" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B51" t="s">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B55" t="s">
+        <v>93</v>
+      </c>
+      <c r="C55" t="s">
         <v>52</v>
       </c>
-      <c r="C51" t="s">
-        <v>52</v>
-      </c>
-      <c r="D51" t="s">
+      <c r="D55" t="s">
         <v>33</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D31:F31 D33:E39" xr:uid="{D53BC0CE-42C5-43E4-95BE-2EB49DEBF56B}">
-      <formula1>$A$28:$A$37</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D35:F35 D37:E43" xr:uid="{D53BC0CE-42C5-43E4-95BE-2EB49DEBF56B}">
+      <formula1>$A$29:$A$41</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C31" xr:uid="{70B37298-4E3B-49F8-A28A-901AB02781B6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C35" xr:uid="{70B37298-4E3B-49F8-A28A-901AB02781B6}">
       <formula1>$A$17:$A$25</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Clean rebuild - fix blank page
</commit_message>
<xml_diff>
--- a/Ingredient.xlsx
+++ b/Ingredient.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cheong Hengq\Desktop\Cheong Hengq\Learnings\Python\Meal2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF315159-AF93-4AE4-AC02-CBE0A5881ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C397C41-7068-42EA-A38B-FAB1C63CF78D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{1B3A883A-8798-493A-91E7-EDD802F8FD64}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="94">
   <si>
     <t>Meat / Protein</t>
   </si>
@@ -1207,9 +1207,6 @@
       <c r="D47" t="s">
         <v>53</v>
       </c>
-      <c r="E47" t="s">
-        <v>54</v>
-      </c>
     </row>
     <row r="48" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B48" t="s">

</xml_diff>